<commit_message>
deterministic evalution got updated
</commit_message>
<xml_diff>
--- a/pipeline/outputs/matrix_base_v4_s3_net_vs_finetuned_epoch3_s3_net.xlsx
+++ b/pipeline/outputs/matrix_base_v4_s3_net_vs_finetuned_epoch3_s3_net.xlsx
@@ -947,10 +947,10 @@
         <v>99.75</v>
       </c>
       <c r="L8" t="n">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="M8" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="N8" t="n">
         <v>98.59999999999999</v>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="9">
@@ -1011,10 +1011,10 @@
         <v>98.98999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="M9" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="N9" t="n">
         <v>97.40000000000001</v>
@@ -1058,10 +1058,10 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H10" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I10" t="n">
         <v>98.8</v>
@@ -1075,10 +1075,10 @@
         <v>99.51000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="M10" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="N10" t="n">
         <v>97.3</v>
@@ -1623,33 +1623,33 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>90.29000000000001</v>
+        <v>91.26000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H19" t="n">
         <v>103</v>
       </c>
       <c r="I19" t="n">
-        <v>83</v>
+        <v>84.2</v>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>75.73</v>
+        <v>77.67</v>
       </c>
       <c r="L19" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M19" t="n">
         <v>103</v>
       </c>
       <c r="N19" t="n">
-        <v>66.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
-        <v>-14.56</v>
+        <v>-13.59</v>
       </c>
     </row>
     <row r="20">
@@ -1752,20 +1752,20 @@
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L21" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M21" t="n">
         <v>100</v>
       </c>
       <c r="N21" t="n">
-        <v>43.3</v>
+        <v>44.3</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
@@ -2456,20 +2456,20 @@
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>82.67</v>
+        <v>85.33</v>
       </c>
       <c r="L33" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M33" t="n">
         <v>75</v>
       </c>
       <c r="N33" t="n">
-        <v>72.59999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
-        <v>-1.33</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="34">
@@ -3239,33 +3239,33 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>51.08</v>
+        <v>50.71</v>
       </c>
       <c r="G47" t="n">
         <v>71</v>
       </c>
       <c r="H47" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I47" t="n">
-        <v>42.9</v>
+        <v>42.5</v>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>86.25</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="L47" t="n">
         <v>69</v>
       </c>
       <c r="M47" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="N47" t="n">
-        <v>77</v>
+        <v>74.7</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
-        <v>35.17</v>
+        <v>33.43</v>
       </c>
     </row>
     <row r="48">
@@ -3295,33 +3295,33 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>57.57</v>
+        <v>57.54</v>
       </c>
       <c r="G48" t="n">
         <v>939</v>
       </c>
       <c r="H48" t="n">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="I48" t="n">
-        <v>55.2</v>
+        <v>55.1</v>
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>82.45999999999999</v>
+        <v>82.48999999999999</v>
       </c>
       <c r="L48" t="n">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="M48" t="n">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="N48" t="n">
         <v>80.2</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>24.88</v>
+        <v>24.95</v>
       </c>
     </row>
     <row r="49">
@@ -3364,20 +3364,20 @@
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>91.14</v>
+        <v>91.31999999999999</v>
       </c>
       <c r="L49" t="n">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="M49" t="n">
         <v>1083</v>
       </c>
       <c r="N49" t="n">
-        <v>89.3</v>
+        <v>89.5</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
-        <v>4.43</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="50">
@@ -3823,7 +3823,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>61.7</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="14">
@@ -4159,7 +4159,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>54.6</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="26">
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>85</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="47">
@@ -4831,7 +4831,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>76.8</v>
+        <v>77.40000000000001</v>
       </c>
     </row>
     <row r="50">
@@ -4915,7 +4915,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>82.90000000000001</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>77.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>84.09999999999999</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71">
@@ -5503,7 +5503,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>82.7</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="74">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>82.40000000000001</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="77">

</xml_diff>